<commit_message>
modified bom to remove spares
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jay_lchicken/PycharmProjects/AudioBox/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E1DCBB9-A725-BB4B-9892-9D11C63D9ABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82A5BA5B-4152-B84C-9B5D-F827BE977B25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="17160" xr2:uid="{0727E5B4-7DFC-874D-AF61-38336D799FD3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Item</t>
   </si>
@@ -69,6 +69,15 @@
   </si>
   <si>
     <t>Seeed Xiao RP2040</t>
+  </si>
+  <si>
+    <t>https://shopee.sg/Stat-2Pcs-Notebook-Speaker-2030-Oval-Loudspeaker-8%CE%A9-1W-Black-Speaker-2-2-kHz-Frequency-Response-Wired-DIY-Accessory-i.110641297.24802861026?extraParams=%7B%22display_model_id%22%3A250076347282%2C%22model_selection_logic%22%3A3%7D&amp;sp_atk=6ad6e27a-c774-49f2-a037-cc04a2b6b14a&amp;xptdk=6ad6e27a-c774-49f2-a037-cc04a2b6b14a</t>
+  </si>
+  <si>
+    <t>https://shopee.sg/1PCS-Microswitch-SS-5-SS-5GL-SS-5GL2-SS-5GL13-SS-5GL-F-SS-5GL2-F-SS-5-F-SS-10GL-SS-01GL13-SS-5GL111-Switch-i.889094752.18895938902?extraParams=%7B%22display_model_id%22%3A250095595431%2C%22model_selection_logic%22%3A3%7D&amp;sp_atk=67b2d27e-e993-4964-acf6-19a2949c651d&amp;xptdk=67b2d27e-e993-4964-acf6-19a2949c651d</t>
+  </si>
+  <si>
+    <t>https://www.seeedstudio.com/XIAO-RP2040-v1-0-p-5026.html</t>
   </si>
 </sst>
 </file>
@@ -128,15 +137,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>990600</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>82636</xdr:rowOff>
+      <xdr:colOff>6870700</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>95336</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>5588000</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>99373</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>647700</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>112073</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -159,7 +168,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5943600" y="692236"/>
+          <a:off x="11823700" y="1720936"/>
           <a:ext cx="4597400" cy="2455137"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -172,15 +181,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>647700</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>69370</xdr:rowOff>
+      <xdr:colOff>7226300</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>82070</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>4914900</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>149404</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>673100</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>162104</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -203,7 +212,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5600700" y="3726970"/>
+          <a:off x="12179300" y="5162070"/>
           <a:ext cx="4267200" cy="1908834"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -577,14 +586,17 @@
         <v>6</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3">
         <v>2.2999999999999998</v>
       </c>
       <c r="D3">
         <f t="shared" ref="D3:D16" si="0">B3*C3</f>
-        <v>4.5999999999999996</v>
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -592,14 +604,17 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4">
         <v>1.6</v>
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>3.2</v>
+        <v>1.6</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -616,6 +631,9 @@
         <f t="shared" si="0"/>
         <v>3.71</v>
       </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D6">
@@ -689,7 +707,7 @@
       </c>
       <c r="D17">
         <f>SUM(D2:D16)</f>
-        <v>48.530000000000008</v>
+        <v>44.63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>